<commit_message>
ScoutTools F-O-S-D Change to sort by DOB only
</commit_message>
<xml_diff>
--- a/scout-tools/format-osm-scout-details/reference_files/example_output.xlsx
+++ b/scout-tools/format-osm-scout-details/reference_files/example_output.xlsx
@@ -506,40 +506,40 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Oliver Bennett</t>
+          <t>Jack Thompson</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>02-11-2013</t>
+          <t>30-01-2013</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Foxes</t>
+          <t>Badgers</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>22 Elm Street, Bristol, BS7 9QW</t>
+          <t>9 Birch Avenue, Bristol, BS5 4GH</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Helen Bennett (Mum) 07700 900221</t>
+          <t>Emma Thompson (Mum) 0117 900 4444</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Allergies: Peanuts - carries EpiPen | Dietary: No nuts | Surgery Medical Info: Confirmed anaphylaxis to peanuts - see care plan on file | Surgery Dietary Needs: Strict nut-free, EpiPen in bag</t>
+          <t>Medical: ADHD - takes medication at breakfast and lunch</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -552,12 +552,12 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Amelia Clarke (Millie)</t>
+          <t>Oliver Bennett</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>12-03-2014</t>
+          <t>02-11-2013</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -565,32 +565,27 @@
           <t>Foxes</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>14 Willow Grove, Bristol, BS8 2AB</t>
+          <t>22 Elm Street, Bristol, BS7 9QW</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Sarah Clarke (Mum) 07700 900111
-David Clarke (Dad) 07700 900112 / 0117 900 2222</t>
+          <t>Helen Bennett (Mum) 07700 900221</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Medical: Mild asthma, carries inhaler | Other: Nervous around dogs</t>
+          <t>Allergies: Peanuts - carries EpiPen | Dietary: No nuts | Surgery Medical Info: Confirmed anaphylaxis to peanuts - see care plan on file | Surgery Dietary Needs: Strict nut-free, EpiPen in bag</t>
         </is>
       </c>
       <c r="B5" s="7" t="n"/>
@@ -603,28 +598,33 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Jack Thompson</t>
+          <t>Amelia Clarke (Millie)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>30-01-2013</t>
+          <t>12-03-2014</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Badgers</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
+          <t>Foxes</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>9 Birch Avenue, Bristol, BS5 4GH</t>
+          <t>14 Willow Grove, Bristol, BS8 2AB</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Emma Thompson (Mum) 0117 900 4444</t>
+          <t>Sarah Clarke (Mum) 07700 900111
+David Clarke (Dad) 07700 900112 / 0117 900 2222</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Medical: ADHD - takes medication at breakfast and lunch</t>
+          <t>Medical: Mild asthma, carries inhaler | Other: Nervous around dogs</t>
         </is>
       </c>
       <c r="B7" s="4" t="n"/>

</xml_diff>